<commit_message>
did a whole pipeline
</commit_message>
<xml_diff>
--- a/data/database/shopgraph_purchase_history copy.xlsx
+++ b/data/database/shopgraph_purchase_history copy.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Manager" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imported Receipts" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP w1_Aug 26" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Purchase History'!$A$1:$S$122</definedName>
@@ -34,7 +35,7 @@
     <numFmt numFmtId="169" formatCode="mmm yyyy"/>
     <numFmt numFmtId="170" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -123,6 +124,14 @@
     <font>
       <b val="1"/>
       <color rgb="001F4E78"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="40">
@@ -364,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -550,6 +559,9 @@
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,7 +640,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -3188,9 +3199,159 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Budget Burndown</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'BP w1_Aug 26'!M1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'BP w1_Aug 26'!$L$2:$L$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'BP w1_Aug 26'!$M$2:$M$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'BP w1_Aug 26'!N1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'BP w1_Aug 26'!$L$2:$L$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'BP w1_Aug 26'!$N$2:$N$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Remaining Budget</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3597,7 +3758,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3780,7 +3940,6 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4136,7 +4295,6 @@
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4389,7 +4547,6 @@
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
   <chart>
     <title>
       <tx>
@@ -4629,7 +4786,6 @@
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -6381,6 +6537,33 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4680000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -19901,8 +20084,8 @@
     <mergeCell ref="Y59:AG62"/>
     <mergeCell ref="S112:V112"/>
     <mergeCell ref="Y142:AG142"/>
+    <mergeCell ref="S146:V146"/>
     <mergeCell ref="S317:V317"/>
-    <mergeCell ref="S146:V146"/>
     <mergeCell ref="Y114:AG114"/>
     <mergeCell ref="S99:V99"/>
     <mergeCell ref="S151:V151"/>
@@ -24672,4 +24855,288 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" style="41" min="1" max="1"/>
+    <col width="48" customWidth="1" style="41" min="2" max="2"/>
+    <col width="22" customWidth="1" style="41" min="12" max="12"/>
+    <col width="22" customWidth="1" style="41" min="13" max="13"/>
+    <col width="22" customWidth="1" style="41" min="14" max="14"/>
+    <col width="22" customWidth="1" style="41" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="89" t="inlineStr">
+        <is>
+          <t>w1_Aug</t>
+        </is>
+      </c>
+      <c r="L1" s="85" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="M1" s="85" t="inlineStr">
+        <is>
+          <t>Ideal Remaining Budget</t>
+        </is>
+      </c>
+      <c r="N1" s="85" t="inlineStr">
+        <is>
+          <t>Actual Remaining Budget</t>
+        </is>
+      </c>
+      <c r="O1" s="85" t="inlineStr">
+        <is>
+          <t>Cumulative Spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="L2" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="M2" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="N2" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O2" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="90" t="inlineStr">
+        <is>
+          <t>Budget Plan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>w1_Aug</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M3" s="87" t="n">
+        <v>233.3333333333333</v>
+      </c>
+      <c r="N3" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O3" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="90" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="M4" s="87" t="n">
+        <v>186.6666666666667</v>
+      </c>
+      <c r="N4" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O4" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="90" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="M5" s="87" t="n">
+        <v>140</v>
+      </c>
+      <c r="N5" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O5" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="90" t="inlineStr">
+        <is>
+          <t>Category Scope</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>All Categories</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="M6" s="87" t="n">
+        <v>93.33333333333334</v>
+      </c>
+      <c r="N6" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O6" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="90" t="inlineStr">
+        <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>All Categories</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="M7" s="87" t="n">
+        <v>46.66666666666666</v>
+      </c>
+      <c r="N7" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O7" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="90" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="M8" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="87" t="n">
+        <v>280</v>
+      </c>
+      <c r="O8" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="90" t="inlineStr">
+        <is>
+          <t>Total Spent</t>
+        </is>
+      </c>
+      <c r="B9" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="90" t="inlineStr">
+        <is>
+          <t>Remaining Budget</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="90" t="inlineStr">
+        <is>
+          <t>Relevant Date</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="90" t="inlineStr">
+        <is>
+          <t>Ideal Spending Through Relevant Date</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>Actual Spending Through Relevant Date</t>
+        </is>
+      </c>
+      <c r="B13" s="87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="90" t="inlineStr">
+        <is>
+          <t>Ahead / Behind Budget</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>On pace</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="91" t="inlineStr">
+        <is>
+          <t>Budget Burndown</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="40" t="inlineStr">
+        <is>
+          <t>Interpretation: Actual Remaining above Ideal Remaining means spending is running below the planned burn rate. Below the ideal line means spending is running above the planned burn rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A47:H49"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>